<commit_message>
Refactor Home Finder Playwright framework
</commit_message>
<xml_diff>
--- a/src/resources/data/ReferNest_Testdata_6_Cities.xlsx
+++ b/src/resources/data/ReferNest_Testdata_6_Cities.xlsx
@@ -5,6 +5,9 @@
   <sheets>
     <sheet name="Refer" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Refer'!A1:AA7</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AB7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,7 +422,7 @@
         <v>preferred_tenants</v>
       </c>
       <c r="G1" t="str">
-        <v xml:space="preserve">street_address </v>
+        <v>street_address</v>
       </c>
       <c r="H1" t="str">
         <v>building_details</v>
@@ -428,7 +431,7 @@
         <v>landmark</v>
       </c>
       <c r="J1" t="str">
-        <v xml:space="preserve">monthly_rent </v>
+        <v>monthly_rent</v>
       </c>
       <c r="K1" t="str">
         <v>security_deposit</v>
@@ -480,6 +483,9 @@
       </c>
       <c r="AA1" t="str">
         <v>property_photos</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>status</v>
       </c>
     </row>
     <row r="2">
@@ -564,6 +570,9 @@
       <c r="AA2" t="str">
         <v>No</v>
       </c>
+      <c r="AB2" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -647,6 +656,9 @@
       <c r="AA3" t="str">
         <v>No</v>
       </c>
+      <c r="AB3" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -730,6 +742,9 @@
       <c r="AA4" t="str">
         <v>No</v>
       </c>
+      <c r="AB4" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -813,13 +828,16 @@
       <c r="AA5" t="str">
         <v>No</v>
       </c>
+      <c r="AB5" t="str">
+        <v>Pass</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>TC_006</v>
       </c>
       <c r="B6" t="str">
-        <v>Bangalore</v>
+        <v>Chennai</v>
       </c>
       <c r="C6" t="str">
         <v>Anna Nagar</v>
@@ -895,6 +913,9 @@
       </c>
       <c r="AA6" t="str">
         <v>No</v>
+      </c>
+      <c r="AB6" t="str">
+        <v>Pass</v>
       </c>
     </row>
     <row r="7">
@@ -979,11 +1000,15 @@
       <c r="AA7" t="str">
         <v>No</v>
       </c>
+      <c r="AB7" t="str">
+        <v>Pass</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AA7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>